<commit_message>
Add new transaction Excel files and update existing ones
- Updated existing transaction Excel files to reflect recent changes.
- Added two new Excel files (3.xlsx and 5.xlsx) to enhance the dataset for transaction processing and analysis.
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 1.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{969D4BF4-1156-4077-8B7C-20B77F265EC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F17E75-5177-4F45-9830-F7BFFDB44499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6991,7 +6991,7 @@
         <v>138</v>
       </c>
       <c r="B143" s="17" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C143" s="12" t="s">
         <v>166</v>
@@ -7029,7 +7029,7 @@
         <v>139</v>
       </c>
       <c r="B144" s="17" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C144" s="12" t="s">
         <v>167</v>

</xml_diff>

<commit_message>
Update existing transaction Excel files to reflect recent changes
- Modified two existing Excel files (1.xlsx and 2.xlsx) to incorporate updated transaction data.
- Ensured consistency and accuracy in the dataset for improved analysis and reporting.
</commit_message>
<xml_diff>
--- a/data/transactions/أذونات الإضافة لشهر 1.xlsx
+++ b/data/transactions/أذونات الإضافة لشهر 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ERP\erp-server\data\transactions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07F17E75-5177-4F45-9830-F7BFFDB44499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68045AA6-26F4-41AE-95E8-FD4A87E4FA89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1024" uniqueCount="355">
   <si>
     <t>بورسعيد لصناعة المعادن</t>
   </si>
@@ -291,9 +291,6 @@
     <t xml:space="preserve">محبس 1بوصه SST </t>
   </si>
   <si>
-    <t>الراضوان</t>
-  </si>
-  <si>
     <t xml:space="preserve">كوع 1 بوصه SST </t>
   </si>
   <si>
@@ -321,9 +318,6 @@
     <t>طقم مجري بلوم 50 سم ظهر 18</t>
   </si>
   <si>
-    <t>ماران انا</t>
-  </si>
-  <si>
     <t>سلونيت مياه 1/2</t>
   </si>
   <si>
@@ -423,9 +417,6 @@
     <t>15/1/2026</t>
   </si>
   <si>
-    <t>البعلبكي</t>
-  </si>
-  <si>
     <t xml:space="preserve">برميل بوليو </t>
   </si>
   <si>
@@ -1105,6 +1096,12 @@
   </si>
   <si>
     <t>25/1/2026</t>
+  </si>
+  <si>
+    <t>ماران اثا</t>
+  </si>
+  <si>
+    <t>البعلبلكي</t>
   </si>
 </sst>
 </file>
@@ -1731,14 +1728,14 @@
   <cols>
     <col min="1" max="1" width="6.5703125" customWidth="1"/>
     <col min="2" max="2" width="16.5703125" customWidth="1"/>
-    <col min="3" max="3" width="31.28515625" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" customWidth="1"/>
+    <col min="3" max="3" width="46.5703125" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" customWidth="1"/>
     <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.85546875" customWidth="1"/>
     <col min="7" max="7" width="15.28515625" customWidth="1"/>
     <col min="8" max="8" width="13.28515625" customWidth="1"/>
     <col min="9" max="9" width="18.7109375" customWidth="1"/>
-    <col min="10" max="10" width="23.140625" customWidth="1"/>
+    <col min="10" max="10" width="30.140625" customWidth="1"/>
     <col min="11" max="11" width="14.85546875" customWidth="1"/>
     <col min="12" max="12" width="15.140625" customWidth="1"/>
   </cols>
@@ -1821,7 +1818,7 @@
         <v>1</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>20</v>
@@ -1859,7 +1856,7 @@
         <v>2</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>21</v>
@@ -1897,7 +1894,7 @@
         <v>3</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>23</v>
@@ -1935,7 +1932,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>27</v>
@@ -1973,7 +1970,7 @@
         <v>5</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>28</v>
@@ -2011,7 +2008,7 @@
         <v>6</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>29</v>
@@ -2049,7 +2046,7 @@
         <v>7</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>30</v>
@@ -2087,7 +2084,7 @@
         <v>8</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>31</v>
@@ -2127,7 +2124,7 @@
         <v>9</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>32</v>
@@ -2165,7 +2162,7 @@
         <v>10</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>33</v>
@@ -2203,7 +2200,7 @@
         <v>11</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>34</v>
@@ -2241,7 +2238,7 @@
         <v>12</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>35</v>
@@ -2279,7 +2276,7 @@
         <v>13</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>36</v>
@@ -2317,7 +2314,7 @@
         <v>14</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>37</v>
@@ -2355,7 +2352,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="25" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>38</v>
@@ -2393,7 +2390,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C22" s="11" t="s">
         <v>41</v>
@@ -2431,7 +2428,7 @@
         <v>17</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>42</v>
@@ -2469,7 +2466,7 @@
         <v>18</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>45</v>
@@ -2507,7 +2504,7 @@
         <v>19</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C25" s="11" t="s">
         <v>64</v>
@@ -2545,7 +2542,7 @@
         <v>20</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>46</v>
@@ -2583,7 +2580,7 @@
         <v>21</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>65</v>
@@ -2621,7 +2618,7 @@
         <v>23</v>
       </c>
       <c r="B28" s="25" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>51</v>
@@ -2659,7 +2656,7 @@
         <v>24</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>66</v>
@@ -2697,7 +2694,7 @@
         <v>25</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>53</v>
@@ -2735,7 +2732,7 @@
         <v>26</v>
       </c>
       <c r="B31" s="17" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>55</v>
@@ -2773,7 +2770,7 @@
         <v>27</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>56</v>
@@ -2811,7 +2808,7 @@
         <v>28</v>
       </c>
       <c r="B33" s="17" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>57</v>
@@ -2849,7 +2846,7 @@
         <v>29</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>58</v>
@@ -2887,7 +2884,7 @@
         <v>30</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>59</v>
@@ -2925,7 +2922,7 @@
         <v>31</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>60</v>
@@ -2963,7 +2960,7 @@
         <v>32</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>61</v>
@@ -3001,7 +2998,7 @@
         <v>33</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>62</v>
@@ -3039,7 +3036,7 @@
         <v>34</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>63</v>
@@ -3077,7 +3074,7 @@
         <v>35</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>67</v>
@@ -3115,7 +3112,7 @@
         <v>36</v>
       </c>
       <c r="B41" s="26" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C41" s="11" t="s">
         <v>68</v>
@@ -3153,7 +3150,7 @@
         <v>37</v>
       </c>
       <c r="B42" s="26" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C42" s="11" t="s">
         <v>69</v>
@@ -3191,7 +3188,7 @@
         <v>38</v>
       </c>
       <c r="B43" s="26" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C43" s="11" t="s">
         <v>70</v>
@@ -3229,7 +3226,7 @@
         <v>39</v>
       </c>
       <c r="B44" s="26" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C44" s="11" t="s">
         <v>71</v>
@@ -3267,7 +3264,7 @@
         <v>40</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C45" s="11" t="s">
         <v>72</v>
@@ -3305,7 +3302,7 @@
         <v>41</v>
       </c>
       <c r="B46" s="17" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C46" s="11" t="s">
         <v>74</v>
@@ -3343,7 +3340,7 @@
         <v>42</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C47" s="11" t="s">
         <v>75</v>
@@ -3381,7 +3378,7 @@
         <v>43</v>
       </c>
       <c r="B48" s="17" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C48" s="11" t="s">
         <v>76</v>
@@ -3419,7 +3416,7 @@
         <v>44</v>
       </c>
       <c r="B49" s="17" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C49" s="11" t="s">
         <v>77</v>
@@ -3457,7 +3454,7 @@
         <v>45</v>
       </c>
       <c r="B50" s="17" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C50" s="11" t="s">
         <v>78</v>
@@ -3495,7 +3492,7 @@
         <v>46</v>
       </c>
       <c r="B51" s="17" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C51" s="11" t="s">
         <v>79</v>
@@ -3533,7 +3530,7 @@
         <v>47</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C52" s="11" t="s">
         <v>80</v>
@@ -3571,7 +3568,7 @@
         <v>48</v>
       </c>
       <c r="B53" s="17" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="C53" s="11" t="s">
         <v>81</v>
@@ -3609,10 +3606,10 @@
         <v>49</v>
       </c>
       <c r="B54" s="17" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D54" s="11" t="s">
         <v>24</v>
@@ -3647,7 +3644,7 @@
         <v>50</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C55" s="12" t="s">
         <v>83</v>
@@ -3671,7 +3668,7 @@
         <v>46357</v>
       </c>
       <c r="J55" s="12" t="s">
-        <v>84</v>
+        <v>128</v>
       </c>
       <c r="K55" s="11">
         <v>6116</v>
@@ -3685,10 +3682,10 @@
         <v>51</v>
       </c>
       <c r="B56" s="17" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D56" s="11" t="s">
         <v>24</v>
@@ -3709,7 +3706,7 @@
         <v>46357</v>
       </c>
       <c r="J56" s="12" t="s">
-        <v>84</v>
+        <v>128</v>
       </c>
       <c r="K56" s="11">
         <v>6116</v>
@@ -3723,10 +3720,10 @@
         <v>52</v>
       </c>
       <c r="B57" s="17" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C57" s="27" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D57" s="11" t="s">
         <v>24</v>
@@ -3747,7 +3744,7 @@
         <v>46357</v>
       </c>
       <c r="J57" s="12" t="s">
-        <v>84</v>
+        <v>128</v>
       </c>
       <c r="K57" s="11">
         <v>6116</v>
@@ -3761,10 +3758,10 @@
         <v>53</v>
       </c>
       <c r="B58" s="17" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D58" s="11" t="s">
         <v>24</v>
@@ -3799,10 +3796,10 @@
         <v>54</v>
       </c>
       <c r="B59" s="17" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D59" s="11" t="s">
         <v>24</v>
@@ -3837,10 +3834,10 @@
         <v>55</v>
       </c>
       <c r="B60" s="17" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="C60" s="12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D60" s="11" t="s">
         <v>24</v>
@@ -3858,10 +3855,10 @@
         <v>754</v>
       </c>
       <c r="I60" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="J60" s="12" t="s">
         <v>90</v>
-      </c>
-      <c r="J60" s="12" t="s">
-        <v>91</v>
       </c>
       <c r="K60" s="11">
         <v>6118</v>
@@ -3875,10 +3872,10 @@
         <v>56</v>
       </c>
       <c r="B61" s="17" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D61" s="11" t="s">
         <v>24</v>
@@ -3896,10 +3893,10 @@
         <v>1</v>
       </c>
       <c r="I61" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J61" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K61" s="11">
         <v>6119</v>
@@ -3913,10 +3910,10 @@
         <v>57</v>
       </c>
       <c r="B62" s="17" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D62" s="11" t="s">
         <v>24</v>
@@ -3934,10 +3931,10 @@
         <v>1</v>
       </c>
       <c r="I62" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J62" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K62" s="11">
         <v>6119</v>
@@ -3951,10 +3948,10 @@
         <v>58</v>
       </c>
       <c r="B63" s="25" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D63" s="11" t="s">
         <v>24</v>
@@ -3972,10 +3969,10 @@
         <v>2</v>
       </c>
       <c r="I63" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J63" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K63" s="11">
         <v>6120</v>
@@ -3989,10 +3986,10 @@
         <v>59</v>
       </c>
       <c r="B64" s="17" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D64" s="11" t="s">
         <v>24</v>
@@ -4010,10 +4007,10 @@
         <v>2</v>
       </c>
       <c r="I64" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J64" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K64" s="11">
         <v>6120</v>
@@ -4027,10 +4024,10 @@
         <v>60</v>
       </c>
       <c r="B65" s="25" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D65" s="11" t="s">
         <v>24</v>
@@ -4048,10 +4045,10 @@
         <v>3</v>
       </c>
       <c r="I65" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J65" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K65" s="11">
         <v>6121</v>
@@ -4065,10 +4062,10 @@
         <v>61</v>
       </c>
       <c r="B66" s="29" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D66" s="11" t="s">
         <v>24</v>
@@ -4086,10 +4083,10 @@
         <v>3</v>
       </c>
       <c r="I66" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J66" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K66" s="11">
         <v>6121</v>
@@ -4103,10 +4100,10 @@
         <v>62</v>
       </c>
       <c r="B67" s="29" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D67" s="11" t="s">
         <v>24</v>
@@ -4124,10 +4121,10 @@
         <v>3</v>
       </c>
       <c r="I67" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J67" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K67" s="11">
         <v>6121</v>
@@ -4141,10 +4138,10 @@
         <v>63</v>
       </c>
       <c r="B68" s="25" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D68" s="11" t="s">
         <v>24</v>
@@ -4162,10 +4159,10 @@
         <v>3</v>
       </c>
       <c r="I68" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J68" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K68" s="11">
         <v>6121</v>
@@ -4179,10 +4176,10 @@
         <v>64</v>
       </c>
       <c r="B69" s="17" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="D69" s="11" t="s">
         <v>24</v>
@@ -4200,10 +4197,10 @@
         <v>3</v>
       </c>
       <c r="I69" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="J69" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K69" s="11">
         <v>6121</v>
@@ -4217,10 +4214,10 @@
         <v>65</v>
       </c>
       <c r="B70" s="29" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D70" s="11" t="s">
         <v>24</v>
@@ -4238,7 +4235,7 @@
         <v>2426</v>
       </c>
       <c r="I70" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J70" s="12" t="s">
         <v>49</v>
@@ -4255,10 +4252,10 @@
         <v>66</v>
       </c>
       <c r="B71" s="26" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D71" s="11" t="s">
         <v>24</v>
@@ -4276,7 +4273,7 @@
         <v>2426</v>
       </c>
       <c r="I71" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J71" s="12" t="s">
         <v>49</v>
@@ -4293,10 +4290,10 @@
         <v>67</v>
       </c>
       <c r="B72" s="26" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D72" s="11" t="s">
         <v>24</v>
@@ -4314,7 +4311,7 @@
         <v>2426</v>
       </c>
       <c r="I72" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J72" s="12" t="s">
         <v>49</v>
@@ -4331,10 +4328,10 @@
         <v>68</v>
       </c>
       <c r="B73" s="29" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D73" s="11" t="s">
         <v>24</v>
@@ -4352,7 +4349,7 @@
         <v>2426</v>
       </c>
       <c r="I73" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J73" s="12" t="s">
         <v>49</v>
@@ -4369,10 +4366,10 @@
         <v>69</v>
       </c>
       <c r="B74" s="25" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="C74" s="12" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D74" s="11" t="s">
         <v>24</v>
@@ -4390,7 +4387,7 @@
         <v>2426</v>
       </c>
       <c r="I74" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J74" s="12" t="s">
         <v>49</v>
@@ -4407,10 +4404,10 @@
         <v>70</v>
       </c>
       <c r="B75" s="25" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C75" s="12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="D75" s="11" t="s">
         <v>24</v>
@@ -4428,7 +4425,7 @@
         <v>2426</v>
       </c>
       <c r="I75" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J75" s="12" t="s">
         <v>49</v>
@@ -4445,10 +4442,10 @@
         <v>71</v>
       </c>
       <c r="B76" s="25" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C76" s="12" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D76" s="11" t="s">
         <v>24</v>
@@ -4466,7 +4463,7 @@
         <v>2426</v>
       </c>
       <c r="I76" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J76" s="12" t="s">
         <v>49</v>
@@ -4483,10 +4480,10 @@
         <v>72</v>
       </c>
       <c r="B77" s="25" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C77" s="12" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D77" s="11" t="s">
         <v>24</v>
@@ -4504,7 +4501,7 @@
         <v>2426</v>
       </c>
       <c r="I77" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J77" s="12" t="s">
         <v>49</v>
@@ -4521,10 +4518,10 @@
         <v>73</v>
       </c>
       <c r="B78" s="29" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="C78" s="12" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="D78" s="11" t="s">
         <v>24</v>
@@ -4542,7 +4539,7 @@
         <v>2426</v>
       </c>
       <c r="I78" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J78" s="12" t="s">
         <v>49</v>
@@ -4559,10 +4556,10 @@
         <v>74</v>
       </c>
       <c r="B79" s="25" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C79" s="12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="D79" s="11" t="s">
         <v>24</v>
@@ -4580,7 +4577,7 @@
         <v>2426</v>
       </c>
       <c r="I79" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J79" s="12" t="s">
         <v>49</v>
@@ -4597,10 +4594,10 @@
         <v>75</v>
       </c>
       <c r="B80" s="17" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="C80" s="12" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D80" s="11" t="s">
         <v>24</v>
@@ -4618,7 +4615,7 @@
         <v>2426</v>
       </c>
       <c r="I80" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J80" s="12" t="s">
         <v>49</v>
@@ -4635,10 +4632,10 @@
         <v>76</v>
       </c>
       <c r="B81" s="17" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C81" s="12" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D81" s="11" t="s">
         <v>24</v>
@@ -4656,7 +4653,7 @@
         <v>2426</v>
       </c>
       <c r="I81" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J81" s="12" t="s">
         <v>49</v>
@@ -4673,10 +4670,10 @@
         <v>77</v>
       </c>
       <c r="B82" s="29" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="C82" s="12" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D82" s="11" t="s">
         <v>24</v>
@@ -4694,7 +4691,7 @@
         <v>2426</v>
       </c>
       <c r="I82" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J82" s="12" t="s">
         <v>49</v>
@@ -4711,10 +4708,10 @@
         <v>78</v>
       </c>
       <c r="B83" s="29" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C83" s="12" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D83" s="11" t="s">
         <v>24</v>
@@ -4732,7 +4729,7 @@
         <v>2426</v>
       </c>
       <c r="I83" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J83" s="12" t="s">
         <v>49</v>
@@ -4749,10 +4746,10 @@
         <v>79</v>
       </c>
       <c r="B84" s="29" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C84" s="12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D84" s="11" t="s">
         <v>24</v>
@@ -4770,7 +4767,7 @@
         <v>2426</v>
       </c>
       <c r="I84" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J84" s="12" t="s">
         <v>49</v>
@@ -4787,10 +4784,10 @@
         <v>80</v>
       </c>
       <c r="B85" s="29" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C85" s="12" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D85" s="11" t="s">
         <v>24</v>
@@ -4808,7 +4805,7 @@
         <v>2426</v>
       </c>
       <c r="I85" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J85" s="12" t="s">
         <v>49</v>
@@ -4825,10 +4822,10 @@
         <v>81</v>
       </c>
       <c r="B86" s="29" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C86" s="12" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D86" s="11" t="s">
         <v>24</v>
@@ -4846,7 +4843,7 @@
         <v>2426</v>
       </c>
       <c r="I86" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J86" s="12" t="s">
         <v>49</v>
@@ -4863,10 +4860,10 @@
         <v>82</v>
       </c>
       <c r="B87" s="29" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C87" s="12" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D87" s="11" t="s">
         <v>24</v>
@@ -4884,7 +4881,7 @@
         <v>2426</v>
       </c>
       <c r="I87" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J87" s="12" t="s">
         <v>49</v>
@@ -4901,10 +4898,10 @@
         <v>83</v>
       </c>
       <c r="B88" s="17" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="C88" s="12" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D88" s="11" t="s">
         <v>24</v>
@@ -4922,10 +4919,10 @@
         <v>12</v>
       </c>
       <c r="I88" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J88" s="12" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="K88" s="11">
         <v>6124</v>
@@ -4939,7 +4936,7 @@
         <v>84</v>
       </c>
       <c r="B89" s="17" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C89" s="12" t="s">
         <v>67</v>
@@ -4960,7 +4957,7 @@
         <v>5055</v>
       </c>
       <c r="I89" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J89" s="12" t="s">
         <v>52</v>
@@ -4977,10 +4974,10 @@
         <v>85</v>
       </c>
       <c r="B90" s="17" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C90" s="12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D90" s="11" t="s">
         <v>24</v>
@@ -4998,16 +4995,16 @@
         <v>13589</v>
       </c>
       <c r="I90" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J90" s="12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K90" s="11">
         <v>6127</v>
       </c>
       <c r="L90" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="91" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5015,10 +5012,10 @@
         <v>86</v>
       </c>
       <c r="B91" s="17" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C91" s="12" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D91" s="11" t="s">
         <v>24</v>
@@ -5036,16 +5033,16 @@
         <v>13589</v>
       </c>
       <c r="I91" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J91" s="12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K91" s="11">
         <v>6127</v>
       </c>
       <c r="L91" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="92" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5053,10 +5050,10 @@
         <v>87</v>
       </c>
       <c r="B92" s="17" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C92" s="12" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D92" s="11" t="s">
         <v>47</v>
@@ -5074,16 +5071,16 @@
         <v>13589</v>
       </c>
       <c r="I92" s="16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J92" s="12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K92" s="11">
         <v>6127</v>
       </c>
       <c r="L92" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="93" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5091,10 +5088,10 @@
         <v>88</v>
       </c>
       <c r="B93" s="17" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C93" s="12" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D93" s="11" t="s">
         <v>47</v>
@@ -5112,16 +5109,16 @@
         <v>173</v>
       </c>
       <c r="I93" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J93" s="12" t="s">
-        <v>128</v>
+        <v>354</v>
       </c>
       <c r="K93" s="11">
         <v>6128</v>
       </c>
       <c r="L93" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="94" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5129,10 +5126,10 @@
         <v>89</v>
       </c>
       <c r="B94" s="17" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C94" s="12" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D94" s="11" t="s">
         <v>47</v>
@@ -5150,16 +5147,16 @@
         <v>173</v>
       </c>
       <c r="I94" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J94" s="12" t="s">
-        <v>128</v>
+        <v>354</v>
       </c>
       <c r="K94" s="11">
         <v>6128</v>
       </c>
       <c r="L94" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="95" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5167,10 +5164,10 @@
         <v>90</v>
       </c>
       <c r="B95" s="17" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="C95" s="12" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D95" s="11" t="s">
         <v>24</v>
@@ -5188,16 +5185,16 @@
         <v>34318</v>
       </c>
       <c r="I95" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J95" s="12" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K95" s="11">
         <v>6129</v>
       </c>
       <c r="L95" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="96" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5205,10 +5202,10 @@
         <v>91</v>
       </c>
       <c r="B96" s="17" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C96" s="12" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D96" s="11" t="s">
         <v>24</v>
@@ -5226,16 +5223,16 @@
         <v>34318</v>
       </c>
       <c r="I96" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J96" s="12" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K96" s="11">
         <v>6129</v>
       </c>
       <c r="L96" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="97" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5243,10 +5240,10 @@
         <v>92</v>
       </c>
       <c r="B97" s="17" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C97" s="12" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D97" s="11" t="s">
         <v>24</v>
@@ -5264,16 +5261,16 @@
         <v>34318</v>
       </c>
       <c r="I97" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J97" s="12" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K97" s="11">
         <v>6129</v>
       </c>
       <c r="L97" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="98" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5281,10 +5278,10 @@
         <v>93</v>
       </c>
       <c r="B98" s="29" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C98" s="12" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="D98" s="11" t="s">
         <v>24</v>
@@ -5302,16 +5299,16 @@
         <v>8</v>
       </c>
       <c r="I98" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J98" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K98" s="11">
         <v>6130</v>
       </c>
       <c r="L98" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="99" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5319,10 +5316,10 @@
         <v>94</v>
       </c>
       <c r="B99" s="25" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C99" s="12" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D99" s="11" t="s">
         <v>24</v>
@@ -5340,16 +5337,16 @@
         <v>8</v>
       </c>
       <c r="I99" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J99" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K99" s="11">
         <v>6130</v>
       </c>
       <c r="L99" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="100" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5357,10 +5354,10 @@
         <v>95</v>
       </c>
       <c r="B100" s="25" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="C100" s="12" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D100" s="11" t="s">
         <v>24</v>
@@ -5378,16 +5375,16 @@
         <v>8</v>
       </c>
       <c r="I100" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J100" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K100" s="11">
         <v>6130</v>
       </c>
       <c r="L100" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="101" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5395,10 +5392,10 @@
         <v>96</v>
       </c>
       <c r="B101" s="25" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="C101" s="12" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="D101" s="11" t="s">
         <v>24</v>
@@ -5416,16 +5413,16 @@
         <v>8</v>
       </c>
       <c r="I101" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J101" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K101" s="11">
         <v>6130</v>
       </c>
       <c r="L101" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="102" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5433,10 +5430,10 @@
         <v>97</v>
       </c>
       <c r="B102" s="29" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="C102" s="12" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D102" s="11" t="s">
         <v>24</v>
@@ -5454,16 +5451,16 @@
         <v>8</v>
       </c>
       <c r="I102" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J102" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K102" s="11">
         <v>6130</v>
       </c>
       <c r="L102" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="103" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5471,10 +5468,10 @@
         <v>98</v>
       </c>
       <c r="B103" s="29" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C103" s="12" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D103" s="11" t="s">
         <v>24</v>
@@ -5492,16 +5489,16 @@
         <v>8</v>
       </c>
       <c r="I103" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J103" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K103" s="11">
         <v>6130</v>
       </c>
       <c r="L103" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="104" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5509,10 +5506,10 @@
         <v>99</v>
       </c>
       <c r="B104" s="29" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="C104" s="12" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D104" s="11" t="s">
         <v>24</v>
@@ -5530,16 +5527,16 @@
         <v>8</v>
       </c>
       <c r="I104" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J104" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K104" s="11">
         <v>6130</v>
       </c>
       <c r="L104" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="105" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5547,10 +5544,10 @@
         <v>100</v>
       </c>
       <c r="B105" s="29" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="C105" s="12" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D105" s="11" t="s">
         <v>24</v>
@@ -5568,16 +5565,16 @@
         <v>8</v>
       </c>
       <c r="I105" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J105" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K105" s="11">
         <v>6130</v>
       </c>
       <c r="L105" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="106" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5585,10 +5582,10 @@
         <v>101</v>
       </c>
       <c r="B106" s="29" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C106" s="12" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D106" s="11" t="s">
         <v>24</v>
@@ -5606,16 +5603,16 @@
         <v>8</v>
       </c>
       <c r="I106" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J106" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K106" s="11">
         <v>6130</v>
       </c>
       <c r="L106" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="107" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5623,10 +5620,10 @@
         <v>102</v>
       </c>
       <c r="B107" s="17" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C107" s="12" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D107" s="11" t="s">
         <v>24</v>
@@ -5644,16 +5641,16 @@
         <v>8</v>
       </c>
       <c r="I107" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J107" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K107" s="11">
         <v>6130</v>
       </c>
       <c r="L107" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="108" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5661,10 +5658,10 @@
         <v>103</v>
       </c>
       <c r="B108" s="25" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C108" s="12" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="D108" s="11" t="s">
         <v>24</v>
@@ -5682,16 +5679,16 @@
         <v>8</v>
       </c>
       <c r="I108" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J108" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K108" s="11">
         <v>6130</v>
       </c>
       <c r="L108" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="109" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5699,10 +5696,10 @@
         <v>104</v>
       </c>
       <c r="B109" s="17" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C109" s="12" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D109" s="11" t="s">
         <v>24</v>
@@ -5720,16 +5717,16 @@
         <v>8</v>
       </c>
       <c r="I109" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J109" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K109" s="11">
         <v>6130</v>
       </c>
       <c r="L109" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="110" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5737,10 +5734,10 @@
         <v>105</v>
       </c>
       <c r="B110" s="29" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C110" s="12" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D110" s="11" t="s">
         <v>24</v>
@@ -5758,16 +5755,16 @@
         <v>8</v>
       </c>
       <c r="I110" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J110" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K110" s="11">
         <v>6131</v>
       </c>
       <c r="L110" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="111" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5775,10 +5772,10 @@
         <v>106</v>
       </c>
       <c r="B111" s="29" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C111" s="12" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D111" s="11" t="s">
         <v>24</v>
@@ -5796,16 +5793,16 @@
         <v>8</v>
       </c>
       <c r="I111" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J111" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K111" s="11">
         <v>6131</v>
       </c>
       <c r="L111" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="112" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5813,10 +5810,10 @@
         <v>107</v>
       </c>
       <c r="B112" s="29" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="C112" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D112" s="11" t="s">
         <v>24</v>
@@ -5834,16 +5831,16 @@
         <v>8</v>
       </c>
       <c r="I112" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J112" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K112" s="11">
         <v>6131</v>
       </c>
       <c r="L112" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="113" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5851,10 +5848,10 @@
         <v>108</v>
       </c>
       <c r="B113" s="29" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C113" s="12" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D113" s="11" t="s">
         <v>24</v>
@@ -5872,16 +5869,16 @@
         <v>8</v>
       </c>
       <c r="I113" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J113" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K113" s="11">
         <v>6131</v>
       </c>
       <c r="L113" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="114" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5889,10 +5886,10 @@
         <v>109</v>
       </c>
       <c r="B114" s="29" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C114" s="12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D114" s="11" t="s">
         <v>24</v>
@@ -5910,16 +5907,16 @@
         <v>8</v>
       </c>
       <c r="I114" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J114" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K114" s="11">
         <v>6131</v>
       </c>
       <c r="L114" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="115" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5927,10 +5924,10 @@
         <v>110</v>
       </c>
       <c r="B115" s="17" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="C115" s="12" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D115" s="11" t="s">
         <v>24</v>
@@ -5948,16 +5945,16 @@
         <v>8</v>
       </c>
       <c r="I115" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J115" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K115" s="11">
         <v>6131</v>
       </c>
       <c r="L115" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="116" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -5965,10 +5962,10 @@
         <v>111</v>
       </c>
       <c r="B116" s="25" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="C116" s="12" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D116" s="11" t="s">
         <v>24</v>
@@ -5986,16 +5983,16 @@
         <v>9</v>
       </c>
       <c r="I116" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J116" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K116" s="11">
         <v>6132</v>
       </c>
       <c r="L116" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="117" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6003,10 +6000,10 @@
         <v>112</v>
       </c>
       <c r="B117" s="17" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="C117" s="12" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D117" s="11" t="s">
         <v>24</v>
@@ -6024,16 +6021,16 @@
         <v>9</v>
       </c>
       <c r="I117" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J117" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K117" s="11">
         <v>6132</v>
       </c>
       <c r="L117" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="118" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6041,10 +6038,10 @@
         <v>113</v>
       </c>
       <c r="B118" s="25" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="C118" s="12" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D118" s="11" t="s">
         <v>24</v>
@@ -6062,16 +6059,16 @@
         <v>9</v>
       </c>
       <c r="I118" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J118" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K118" s="11">
         <v>6132</v>
       </c>
       <c r="L118" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="119" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6079,10 +6076,10 @@
         <v>114</v>
       </c>
       <c r="B119" s="17" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C119" s="12" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D119" s="11" t="s">
         <v>24</v>
@@ -6100,16 +6097,16 @@
         <v>9</v>
       </c>
       <c r="I119" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J119" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K119" s="11">
         <v>6132</v>
       </c>
       <c r="L119" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="120" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6117,10 +6114,10 @@
         <v>115</v>
       </c>
       <c r="B120" s="25" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="C120" s="12" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D120" s="11" t="s">
         <v>24</v>
@@ -6138,16 +6135,16 @@
         <v>9</v>
       </c>
       <c r="I120" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J120" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K120" s="11">
         <v>6132</v>
       </c>
       <c r="L120" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="121" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6155,10 +6152,10 @@
         <v>116</v>
       </c>
       <c r="B121" s="17" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C121" s="12" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D121" s="11" t="s">
         <v>24</v>
@@ -6176,16 +6173,16 @@
         <v>9</v>
       </c>
       <c r="I121" s="16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J121" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K121" s="11">
         <v>6132</v>
       </c>
       <c r="L121" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="122" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6193,10 +6190,10 @@
         <v>117</v>
       </c>
       <c r="B122" s="17" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C122" s="12" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D122" s="11" t="s">
         <v>24</v>
@@ -6214,16 +6211,16 @@
         <v>10</v>
       </c>
       <c r="I122" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J122" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K122" s="11">
         <v>6133</v>
       </c>
       <c r="L122" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="123" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6231,10 +6228,10 @@
         <v>118</v>
       </c>
       <c r="B123" s="17" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="C123" s="12" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D123" s="11" t="s">
         <v>24</v>
@@ -6252,16 +6249,16 @@
         <v>10</v>
       </c>
       <c r="I123" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J123" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K123" s="11">
         <v>6133</v>
       </c>
       <c r="L123" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="124" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6269,10 +6266,10 @@
         <v>119</v>
       </c>
       <c r="B124" s="17" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="C124" s="12" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="D124" s="11" t="s">
         <v>24</v>
@@ -6290,16 +6287,16 @@
         <v>10</v>
       </c>
       <c r="I124" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J124" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K124" s="11">
         <v>6133</v>
       </c>
       <c r="L124" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="125" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6307,10 +6304,10 @@
         <v>120</v>
       </c>
       <c r="B125" s="17" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="C125" s="12" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D125" s="11" t="s">
         <v>24</v>
@@ -6328,16 +6325,16 @@
         <v>10</v>
       </c>
       <c r="I125" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J125" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K125" s="11">
         <v>6133</v>
       </c>
       <c r="L125" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="126" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6345,10 +6342,10 @@
         <v>121</v>
       </c>
       <c r="B126" s="17" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C126" s="12" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D126" s="11" t="s">
         <v>24</v>
@@ -6366,16 +6363,16 @@
         <v>10</v>
       </c>
       <c r="I126" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J126" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K126" s="11">
         <v>6133</v>
       </c>
       <c r="L126" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="127" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6383,10 +6380,10 @@
         <v>122</v>
       </c>
       <c r="B127" s="25" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="C127" s="12" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D127" s="11" t="s">
         <v>24</v>
@@ -6404,16 +6401,16 @@
         <v>10</v>
       </c>
       <c r="I127" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J127" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K127" s="11">
         <v>6133</v>
       </c>
       <c r="L127" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="128" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6421,10 +6418,10 @@
         <v>123</v>
       </c>
       <c r="B128" s="17" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C128" s="12" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="D128" s="11" t="s">
         <v>24</v>
@@ -6442,7 +6439,7 @@
         <v>4661</v>
       </c>
       <c r="I128" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J128" s="12" t="s">
         <v>73</v>
@@ -6451,7 +6448,7 @@
         <v>6134</v>
       </c>
       <c r="L128" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="129" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6459,10 +6456,10 @@
         <v>124</v>
       </c>
       <c r="B129" s="17" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="C129" s="12" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="D129" s="11" t="s">
         <v>24</v>
@@ -6480,7 +6477,7 @@
         <v>4661</v>
       </c>
       <c r="I129" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J129" s="12" t="s">
         <v>73</v>
@@ -6489,7 +6486,7 @@
         <v>6134</v>
       </c>
       <c r="L129" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="130" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6497,10 +6494,10 @@
         <v>125</v>
       </c>
       <c r="B130" s="17" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="C130" s="12" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D130" s="11" t="s">
         <v>24</v>
@@ -6518,16 +6515,16 @@
         <v>13616</v>
       </c>
       <c r="I130" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J130" s="12" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K130" s="11">
         <v>6135</v>
       </c>
       <c r="L130" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="131" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6535,10 +6532,10 @@
         <v>126</v>
       </c>
       <c r="B131" s="17" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="C131" s="12" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D131" s="11" t="s">
         <v>24</v>
@@ -6556,16 +6553,16 @@
         <v>13616</v>
       </c>
       <c r="I131" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J131" s="12" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K131" s="11">
         <v>6135</v>
       </c>
       <c r="L131" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="132" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6573,10 +6570,10 @@
         <v>127</v>
       </c>
       <c r="B132" s="17" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="C132" s="12" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D132" s="11" t="s">
         <v>24</v>
@@ -6594,16 +6591,16 @@
         <v>13616</v>
       </c>
       <c r="I132" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J132" s="12" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K132" s="11">
         <v>6135</v>
       </c>
       <c r="L132" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="133" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6611,10 +6608,10 @@
         <v>128</v>
       </c>
       <c r="B133" s="17" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C133" s="12" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D133" s="11" t="s">
         <v>24</v>
@@ -6632,16 +6629,16 @@
         <v>13616</v>
       </c>
       <c r="I133" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J133" s="12" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K133" s="11">
         <v>6135</v>
       </c>
       <c r="L133" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="134" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6649,10 +6646,10 @@
         <v>129</v>
       </c>
       <c r="B134" s="17" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="C134" s="12" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="D134" s="11" t="s">
         <v>24</v>
@@ -6670,16 +6667,16 @@
         <v>13616</v>
       </c>
       <c r="I134" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J134" s="12" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K134" s="11">
         <v>6135</v>
       </c>
       <c r="L134" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="135" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6687,10 +6684,10 @@
         <v>130</v>
       </c>
       <c r="B135" s="17" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="C135" s="12" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D135" s="11" t="s">
         <v>24</v>
@@ -6708,16 +6705,16 @@
         <v>13616</v>
       </c>
       <c r="I135" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J135" s="12" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K135" s="11">
         <v>6135</v>
       </c>
       <c r="L135" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="136" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6725,10 +6722,10 @@
         <v>131</v>
       </c>
       <c r="B136" s="17" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="C136" s="12" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D136" s="11" t="s">
         <v>24</v>
@@ -6746,16 +6743,16 @@
         <v>34326</v>
       </c>
       <c r="I136" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J136" s="12" t="s">
-        <v>84</v>
+        <v>128</v>
       </c>
       <c r="K136" s="11">
         <v>6136</v>
       </c>
       <c r="L136" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="137" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6763,10 +6760,10 @@
         <v>132</v>
       </c>
       <c r="B137" s="17" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C137" s="12" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D137" s="11" t="s">
         <v>24</v>
@@ -6784,16 +6781,16 @@
         <v>34326</v>
       </c>
       <c r="I137" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J137" s="12" t="s">
-        <v>84</v>
+        <v>128</v>
       </c>
       <c r="K137" s="11">
         <v>6136</v>
       </c>
       <c r="L137" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="138" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6801,10 +6798,10 @@
         <v>133</v>
       </c>
       <c r="B138" s="17" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="C138" s="12" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D138" s="11" t="s">
         <v>24</v>
@@ -6822,16 +6819,16 @@
         <v>34326</v>
       </c>
       <c r="I138" s="16" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="J138" s="12" t="s">
-        <v>84</v>
+        <v>128</v>
       </c>
       <c r="K138" s="11">
         <v>6136</v>
       </c>
       <c r="L138" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="139" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6839,7 +6836,7 @@
         <v>134</v>
       </c>
       <c r="B139" s="17" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C139" s="12" t="s">
         <v>77</v>
@@ -6860,7 +6857,7 @@
         <v>40667</v>
       </c>
       <c r="I139" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J139" s="12" t="s">
         <v>73</v>
@@ -6869,7 +6866,7 @@
         <v>6137</v>
       </c>
       <c r="L139" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="140" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6877,10 +6874,10 @@
         <v>135</v>
       </c>
       <c r="B140" s="17" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="C140" s="12" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D140" s="11" t="s">
         <v>24</v>
@@ -6898,7 +6895,7 @@
         <v>40667</v>
       </c>
       <c r="I140" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J140" s="12" t="s">
         <v>73</v>
@@ -6907,7 +6904,7 @@
         <v>6137</v>
       </c>
       <c r="L140" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="141" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6915,10 +6912,10 @@
         <v>136</v>
       </c>
       <c r="B141" s="17" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="C141" s="12" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D141" s="11" t="s">
         <v>24</v>
@@ -6936,16 +6933,16 @@
         <v>14</v>
       </c>
       <c r="I141" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J141" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K141" s="11">
         <v>6138</v>
       </c>
       <c r="L141" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="142" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6953,10 +6950,10 @@
         <v>137</v>
       </c>
       <c r="B142" s="17" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="C142" s="12" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="D142" s="11" t="s">
         <v>24</v>
@@ -6974,16 +6971,16 @@
         <v>14</v>
       </c>
       <c r="I142" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J142" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K142" s="11">
         <v>6138</v>
       </c>
       <c r="L142" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="143" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -6991,10 +6988,10 @@
         <v>138</v>
       </c>
       <c r="B143" s="17" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="C143" s="12" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D143" s="11" t="s">
         <v>24</v>
@@ -7012,16 +7009,16 @@
         <v>14</v>
       </c>
       <c r="I143" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J143" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K143" s="11">
         <v>6138</v>
       </c>
       <c r="L143" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="144" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7029,10 +7026,10 @@
         <v>139</v>
       </c>
       <c r="B144" s="17" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="C144" s="12" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D144" s="11" t="s">
         <v>47</v>
@@ -7050,16 +7047,16 @@
         <v>14</v>
       </c>
       <c r="I144" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J144" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K144" s="11">
         <v>6138</v>
       </c>
       <c r="L144" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="145" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7067,10 +7064,10 @@
         <v>140</v>
       </c>
       <c r="B145" s="25" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C145" s="12" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D145" s="11" t="s">
         <v>24</v>
@@ -7088,16 +7085,16 @@
         <v>14</v>
       </c>
       <c r="I145" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J145" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K145" s="11">
         <v>6138</v>
       </c>
       <c r="L145" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="146" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7105,10 +7102,10 @@
         <v>141</v>
       </c>
       <c r="B146" s="25" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="C146" s="12" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D146" s="11" t="s">
         <v>24</v>
@@ -7126,16 +7123,16 @@
         <v>14</v>
       </c>
       <c r="I146" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J146" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K146" s="11">
         <v>6138</v>
       </c>
       <c r="L146" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="147" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7143,10 +7140,10 @@
         <v>142</v>
       </c>
       <c r="B147" s="17" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C147" s="12" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D147" s="11" t="s">
         <v>24</v>
@@ -7164,7 +7161,7 @@
         <v>1459</v>
       </c>
       <c r="I147" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J147" s="12" t="s">
         <v>49</v>
@@ -7173,7 +7170,7 @@
         <v>6138</v>
       </c>
       <c r="L147" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="148" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7181,10 +7178,10 @@
         <v>143</v>
       </c>
       <c r="B148" s="17" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C148" s="12" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D148" s="11" t="s">
         <v>24</v>
@@ -7202,7 +7199,7 @@
         <v>1459</v>
       </c>
       <c r="I148" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J148" s="12" t="s">
         <v>49</v>
@@ -7211,7 +7208,7 @@
         <v>6138</v>
       </c>
       <c r="L148" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="149" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7219,10 +7216,10 @@
         <v>144</v>
       </c>
       <c r="B149" s="17" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C149" s="12" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D149" s="11" t="s">
         <v>24</v>
@@ -7240,16 +7237,16 @@
         <v>13625</v>
       </c>
       <c r="I149" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J149" s="12" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K149" s="11">
         <v>6140</v>
       </c>
       <c r="L149" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="150" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7257,7 +7254,7 @@
         <v>145</v>
       </c>
       <c r="B150" s="25" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="C150" s="12" t="s">
         <v>38</v>
@@ -7278,7 +7275,7 @@
         <v>117</v>
       </c>
       <c r="I150" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J150" s="12" t="s">
         <v>39</v>
@@ -7287,7 +7284,7 @@
         <v>6141</v>
       </c>
       <c r="L150" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="151" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7295,10 +7292,10 @@
         <v>146</v>
       </c>
       <c r="B151" s="25" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="C151" s="12" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="D151" s="11" t="s">
         <v>24</v>
@@ -7316,7 +7313,7 @@
         <v>117</v>
       </c>
       <c r="I151" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J151" s="12" t="s">
         <v>39</v>
@@ -7325,7 +7322,7 @@
         <v>6141</v>
       </c>
       <c r="L151" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="152" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7333,10 +7330,10 @@
         <v>147</v>
       </c>
       <c r="B152" s="25" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="C152" s="12" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D152" s="11" t="s">
         <v>24</v>
@@ -7354,7 +7351,7 @@
         <v>5081</v>
       </c>
       <c r="I152" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J152" s="12" t="s">
         <v>52</v>
@@ -7363,7 +7360,7 @@
         <v>6142</v>
       </c>
       <c r="L152" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="153" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7371,10 +7368,10 @@
         <v>148</v>
       </c>
       <c r="B153" s="17" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="C153" s="12" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D153" s="11" t="s">
         <v>24</v>
@@ -7392,7 +7389,7 @@
         <v>5081</v>
       </c>
       <c r="I153" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J153" s="12" t="s">
         <v>52</v>
@@ -7401,7 +7398,7 @@
         <v>6142</v>
       </c>
       <c r="L153" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="154" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7409,10 +7406,10 @@
         <v>149</v>
       </c>
       <c r="B154" s="26" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="C154" s="12" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="D154" s="11" t="s">
         <v>24</v>
@@ -7430,7 +7427,7 @@
         <v>5081</v>
       </c>
       <c r="I154" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J154" s="12" t="s">
         <v>52</v>
@@ -7439,7 +7436,7 @@
         <v>6142</v>
       </c>
       <c r="L154" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="155" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7447,10 +7444,10 @@
         <v>150</v>
       </c>
       <c r="B155" s="17" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="C155" s="12" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D155" s="11" t="s">
         <v>24</v>
@@ -7468,7 +7465,7 @@
         <v>693</v>
       </c>
       <c r="I155" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J155" s="12" t="s">
         <v>44</v>
@@ -7477,7 +7474,7 @@
         <v>6143</v>
       </c>
       <c r="L155" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="156" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7485,10 +7482,10 @@
         <v>151</v>
       </c>
       <c r="B156" s="17" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C156" s="12" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D156" s="11" t="s">
         <v>24</v>
@@ -7506,7 +7503,7 @@
         <v>693</v>
       </c>
       <c r="I156" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J156" s="12" t="s">
         <v>44</v>
@@ -7515,7 +7512,7 @@
         <v>6143</v>
       </c>
       <c r="L156" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="157" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7523,10 +7520,10 @@
         <v>152</v>
       </c>
       <c r="B157" s="17" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="C157" s="12" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="D157" s="11" t="s">
         <v>47</v>
@@ -7544,7 +7541,7 @@
         <v>693</v>
       </c>
       <c r="I157" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J157" s="12" t="s">
         <v>44</v>
@@ -7553,7 +7550,7 @@
         <v>6143</v>
       </c>
       <c r="L157" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="158" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7561,10 +7558,10 @@
         <v>153</v>
       </c>
       <c r="B158" s="17" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C158" s="12" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="D158" s="11" t="s">
         <v>24</v>
@@ -7582,7 +7579,7 @@
         <v>693</v>
       </c>
       <c r="I158" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J158" s="12" t="s">
         <v>44</v>
@@ -7591,7 +7588,7 @@
         <v>6143</v>
       </c>
       <c r="L158" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="159" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7599,10 +7596,10 @@
         <v>154</v>
       </c>
       <c r="B159" s="17" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="C159" s="12" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D159" s="11" t="s">
         <v>24</v>
@@ -7620,16 +7617,16 @@
         <v>16</v>
       </c>
       <c r="I159" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J159" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K159" s="11">
         <v>6144</v>
       </c>
       <c r="L159" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="160" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7637,10 +7634,10 @@
         <v>155</v>
       </c>
       <c r="B160" s="17" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="C160" s="12" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D160" s="11" t="s">
         <v>24</v>
@@ -7658,16 +7655,16 @@
         <v>16</v>
       </c>
       <c r="I160" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J160" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K160" s="11">
         <v>6144</v>
       </c>
       <c r="L160" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="161" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7675,10 +7672,10 @@
         <v>156</v>
       </c>
       <c r="B161" s="26" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="C161" s="12" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="D161" s="11" t="s">
         <v>24</v>
@@ -7696,16 +7693,16 @@
         <v>16</v>
       </c>
       <c r="I161" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J161" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K161" s="11">
         <v>6144</v>
       </c>
       <c r="L161" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="162" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7713,10 +7710,10 @@
         <v>157</v>
       </c>
       <c r="B162" s="17" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="C162" s="12" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D162" s="11" t="s">
         <v>24</v>
@@ -7734,16 +7731,16 @@
         <v>16</v>
       </c>
       <c r="I162" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J162" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K162" s="11">
         <v>6144</v>
       </c>
       <c r="L162" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="163" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7751,10 +7748,10 @@
         <v>158</v>
       </c>
       <c r="B163" s="17" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="C163" s="12" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="D163" s="11" t="s">
         <v>24</v>
@@ -7772,16 +7769,16 @@
         <v>16</v>
       </c>
       <c r="I163" s="16" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="J163" s="12" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
       <c r="K163" s="11">
         <v>6144</v>
       </c>
       <c r="L163" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="164" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7789,10 +7786,10 @@
         <v>159</v>
       </c>
       <c r="B164" s="17" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="C164" s="12" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="D164" s="11" t="s">
         <v>24</v>
@@ -7819,7 +7816,7 @@
         <v>6145</v>
       </c>
       <c r="L164" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="165" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7827,10 +7824,10 @@
         <v>160</v>
       </c>
       <c r="B165" s="17" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="C165" s="12" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D165" s="11" t="s">
         <v>24</v>
@@ -7857,7 +7854,7 @@
         <v>6145</v>
       </c>
       <c r="L165" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="166" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7865,10 +7862,10 @@
         <v>161</v>
       </c>
       <c r="B166" s="17" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="C166" s="12" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D166" s="11" t="s">
         <v>24</v>
@@ -7895,7 +7892,7 @@
         <v>6145</v>
       </c>
       <c r="L166" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="167" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7903,10 +7900,10 @@
         <v>162</v>
       </c>
       <c r="B167" s="17" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C167" s="12" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="D167" s="11" t="s">
         <v>24</v>
@@ -7933,7 +7930,7 @@
         <v>6145</v>
       </c>
       <c r="L167" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="168" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7941,10 +7938,10 @@
         <v>163</v>
       </c>
       <c r="B168" s="17" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="C168" s="12" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="D168" s="11" t="s">
         <v>24</v>
@@ -7971,7 +7968,7 @@
         <v>6145</v>
       </c>
       <c r="L168" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="169" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -7979,10 +7976,10 @@
         <v>164</v>
       </c>
       <c r="B169" s="17" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C169" s="12" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D169" s="11" t="s">
         <v>24</v>
@@ -8009,7 +8006,7 @@
         <v>6145</v>
       </c>
       <c r="L169" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="170" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -8017,10 +8014,10 @@
         <v>165</v>
       </c>
       <c r="B170" s="17" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="C170" s="12" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="D170" s="11" t="s">
         <v>24</v>
@@ -8047,7 +8044,7 @@
         <v>6145</v>
       </c>
       <c r="L170" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="171" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -8055,10 +8052,10 @@
         <v>166</v>
       </c>
       <c r="B171" s="17" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="C171" s="12" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D171" s="11" t="s">
         <v>24</v>
@@ -8085,7 +8082,7 @@
         <v>6145</v>
       </c>
       <c r="L171" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="172" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -8093,10 +8090,10 @@
         <v>167</v>
       </c>
       <c r="B172" s="17" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C172" s="12" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="D172" s="11" t="s">
         <v>24</v>
@@ -8123,7 +8120,7 @@
         <v>6146</v>
       </c>
       <c r="L172" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="173" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -8131,10 +8128,10 @@
         <v>168</v>
       </c>
       <c r="B173" s="25" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C173" s="12" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D173" s="11" t="s">
         <v>24</v>
@@ -8161,7 +8158,7 @@
         <v>6147</v>
       </c>
       <c r="L173" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="174" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -8169,10 +8166,10 @@
         <v>169</v>
       </c>
       <c r="B174" s="25" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C174" s="12" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="D174" s="11" t="s">
         <v>24</v>
@@ -8199,7 +8196,7 @@
         <v>6147</v>
       </c>
       <c r="L174" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="175" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -8207,10 +8204,10 @@
         <v>170</v>
       </c>
       <c r="B175" s="25" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="C175" s="12" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="D175" s="11" t="s">
         <v>24</v>
@@ -8237,7 +8234,7 @@
         <v>6147</v>
       </c>
       <c r="L175" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="176" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -8245,10 +8242,10 @@
         <v>171</v>
       </c>
       <c r="B176" s="17" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C176" s="12" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="D176" s="11" t="s">
         <v>24</v>
@@ -8275,7 +8272,7 @@
         <v>6148</v>
       </c>
       <c r="L176" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="177" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -8283,10 +8280,10 @@
         <v>172</v>
       </c>
       <c r="B177" s="17" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C177" s="12" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="D177" s="11" t="s">
         <v>24</v>
@@ -8313,7 +8310,7 @@
         <v>6148</v>
       </c>
       <c r="L177" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="178" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -8321,10 +8318,10 @@
         <v>173</v>
       </c>
       <c r="B178" s="17" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C178" s="12" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="D178" s="11" t="s">
         <v>24</v>
@@ -8351,7 +8348,7 @@
         <v>6148</v>
       </c>
       <c r="L178" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="179" spans="1:12" ht="28.9" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -8359,10 +8356,10 @@
         <v>174</v>
       </c>
       <c r="B179" s="17" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="C179" s="12" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D179" s="11" t="s">
         <v>24</v>
@@ -8389,7 +8386,7 @@
         <v>6148</v>
       </c>
       <c r="L179" s="14" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="180" spans="1:12" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>

</xml_diff>